<commit_message>
changed the ui of whole report
</commit_message>
<xml_diff>
--- a/scans/dmarc.org/reports/report.xlsx
+++ b/scans/dmarc.org/reports/report.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Subdomains'!$A$1:$B$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Live Hosts'!$A$1:$D$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Open Ports'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Open Ports'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Technologies'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DMARC'!$A$1:$H$5</definedName>
   </definedNames>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -588,7 +588,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>lists.dmarc.org</t>
+          <t>wiki.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>test.dmarc.org</t>
+          <t>lists.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>web.dmarc.org</t>
+          <t>ns2.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>stamp.dmarc.org</t>
+          <t>public.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>wiki.dmarc.org</t>
+          <t>staging.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>cdn.dmarc.org</t>
+          <t>stamp.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>dns1.dmarc.org</t>
+          <t>test.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ns2.dmarc.org</t>
+          <t>v3.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>public.dmarc.org</t>
+          <t>cdn.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>staging.dmarc.org</t>
+          <t>dns1.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>v3.dmarc.org</t>
+          <t>web.dmarc.org</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://wiki.dmarc.org</t>
+          <t>https://lists.dmarc.org</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
@@ -788,7 +788,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>https://lists.dmarc.org</t>
+          <t>https://wiki.dmarc.org</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
@@ -813,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -935,12 +935,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>lists.dmarc.org</t>
+          <t>stamp.dmarc.org</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>587</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>submission</t>
+          <t>smtp</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>smtp</t>
+          <t>http; title=stamp.dmarc.org; server=Apache/2.4.55 (FreeBSD) OpenSSL/1.1.1t-freebsd; status=200</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>443</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>http; title=stamp.dmarc.org; server=Apache/2.4.55 (FreeBSD) OpenSSL/1.1.1t-freebsd; status=200</t>
+          <t>https; title=stamp.dmarc.org; server=Apache/2.4.55 (FreeBSD) OpenSSL/1.1.1t-freebsd; status=200</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>443</t>
+          <t>465</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https; title=stamp.dmarc.org; server=Apache/2.4.55 (FreeBSD) OpenSSL/1.1.1t-freebsd; status=200</t>
+          <t>urd</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>stamp.dmarc.org</t>
+          <t>wiki.dmarc.org</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>465</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1038,19 +1038,19 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>urd</t>
+          <t>http; title=Login required - wiki.dmarc.org; server=Apache/2.4.29 (FreeBSD) PHP/7.2.3 OpenSSL/1.0.2u-freebsd; status=200</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>stamp.dmarc.org</t>
+          <t>www.dmarc.org</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>587</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1060,100 +1060,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>submission</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>wiki.dmarc.org</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>TCP</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>http; title=Login required - wiki.dmarc.org; server=Apache/2.4.29 (FreeBSD) PHP/7.2.3 OpenSSL/1.0.2u-freebsd; status=200</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>wiki.dmarc.org</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>443</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>TCP</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>https; title=Login required - wiki.dmarc.org; server=Apache/2.4.29 (FreeBSD) PHP/7.2.3 OpenSSL/1.0.2u-freebsd; status=200</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>www.dmarc.org</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>TCP</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
           <t>http; title=dmarc.org &amp;#8211; Domain Message Authentication Reporting &amp;amp; Conformance; server=Apache/2.4.29 (FreeBSD) PHP/7.2.3 OpenSSL/1.0.2u-freebsd; status=301; redirect=https://dmarc.org/</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>www.dmarc.org</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>443</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>TCP</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>https; title=dmarc.org &amp;#8211; Domain Message Authentication Reporting &amp;amp; Conformance; server=Apache/2.4.29 (FreeBSD) PHP/7.2.3 OpenSSL/1.0.2u-freebsd; status=301; redirect=https://dmarc.org/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D15"/>
+  <autoFilter ref="A1:D11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1218,7 +1130,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://wiki.dmarc.org</t>
+          <t>https://lists.dmarc.org</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1231,7 +1143,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>https://lists.dmarc.org</t>
+          <t>https://wiki.dmarc.org</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1401,7 +1313,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>wiki.dmarc.org</t>
+          <t>lists.dmarc.org</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1443,7 +1355,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>lists.dmarc.org</t>
+          <t>wiki.dmarc.org</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">

</xml_diff>